<commit_message>
feat: implement multivariate copula tail risk engine and credit underwriting memo
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Stress-Testing" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monte Carlo Risk" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Risk &amp; Copula" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -103,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +122,7 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2122,4 +2124,405 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="59" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MULTIVARIATE COPULA TAIL RISK &amp; CREDIT COMMITTEE UNDERWRITING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>1. MULTIVARIATE COPULA RISK COMPARISON (50,000 SIMULATIONS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Model Specification</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Tail Dep. (Lower / Upper)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Mean DSCR</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Median DSCR</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VaR 95% (5th pct)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VaR 99% (1st pct)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>CVaR 99% (Worst 1%)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>P(DSCR &lt; 1.25x)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>P(DSCR &lt; 1.00x)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>CVaR 99% Deficit (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Gaussian Copula (Benchmark)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>0.00 / 0.00 (Independent)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1.36x</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1.34x</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>0.64x</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>0.37x</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>0.26x</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>42.31%</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>21.61%</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>33,906 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Student-t Copula (nu=4)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>0.18 / 0.18 (Symmetric)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1.36x</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1.34x</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>0.64x</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>0.35x</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>0.21x</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>42.11%</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>21.23%</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>36,735 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Clayton Copula (theta=1.8)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>0.68 / 0.00 (Asymmetric Lower)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1.36x</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1.38x</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>0.49x</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>0.17x</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>0.04x</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>40.35%</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>23.23%</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>47,597 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2. UNDERWRITING SCORECARD &amp; DSRA SIZING</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Underwriting Parameter</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Credit Committee Benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Facility Requested (Senior Mortgage)</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>507,500.00 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Total Project CapEx</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>729,000.00 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Senior Loan-to-Value (Total CapEx)</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>69.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Baseline Year 1 DSCR</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>1.34x</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mature Year 3 DSCR</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>1.73x</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Operating Break-Even Occupancy</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>18.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Debt Service Break-Even Occupancy</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>30.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Standard Covenant DSRA (6 Months)</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>21,774.91 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Recommended Copula Tail DSRA (CVaR 99%)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>47,596.85 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Unhedged Deficit under 6-Month DSRA</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>25,821.94 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Credit Committee Recommendation</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>CONDITIONAL APPROVAL (Escrow DSRA + LEADER Grant Pledge)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: reframe model audit engine and expand excel model to 7 tabs
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Stress-Testing" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monte Carlo Risk" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Risk &amp; Copula" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics &amp; Runway" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,7 +59,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +76,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +130,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2525,4 +2533,1633 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="87" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>UNIT ECONOMICS, CONTRIBUTION MARGIN &amp; 24-MONTH MONTHLY CASH RUNWAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>1. UNIT ECONOMICS &amp; CONTRIBUTION MARGIN (USALI STANDARDS)</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>2. RevPAR &amp; TRevPAR PERFORMANCE SCHEDULE (YEARS 1 TO 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Metric / Cost Category</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Operational / Statutory Basis</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Occupancy Rate</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Occupied Days</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Lodging Revenue (€)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Total Revenue (€)</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Revpar (€)</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Trevpar (€)</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Contribution Margin (€)</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>Fixed Burden Coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Daily Gross Revenue @ 100% Occ</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>1,500.00 EUR</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>8 keys: Lodging 975 EUR + F&amp;B 525 EUR</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Year 1 (Ramp-up)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>28.23%</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>100456.2</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>154548</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>52.93</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>125673.28</v>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>1.09x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Variable Costs per Occupied Day</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>280.25 EUR</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>18.7% variable cost ratio</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Year 2 (Stabilized)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>31.36%</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>111618</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>171720</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>38.23</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>58.81</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>139636.98</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>1.21x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - F&amp;B COGS (30% spend)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>157.50 EUR</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>30% of daily F&amp;B turnover</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Year 3 (Mature)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>32.93%</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>117198.9</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>180306</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>40.14</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>61.75</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>146618.83</v>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>1.27x</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - OTA Commissions (60% OTA @ 15%)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>87.75 EUR</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>15% on 60% OTA booking mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Amenities &amp; Guest Supplies</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>35.00 EUR</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Direct consumables per occupied day</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Unit Contribution Margin (Day)</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>1,219.75 EUR</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>81.32% contribution margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Room-Night Unit Margin</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>107.97 EUR</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>79.98% per room-night</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Annual Fixed Overhead (Payroll + OPEX)</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>72,234.00 EUR</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Base operational fixed costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Annual Senior Debt Service</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>43,536.35 EUR</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>15Y French amortization @ 3.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Annual Total Fixed Burden</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>115,770.35 EUR</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Overhead + full debt service</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Operating Break-Even Occupied Days</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>59.2 Days</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>16.2% annual occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Cash Debt Break-Even Occupied Days</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>94.9 Days</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>26.0% annual occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Bank Covenant 1.25x Break-Even Days</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>103.8 Days</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>28.4% annual occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>3. 24-MONTH EMPIRICAL CASH RUNWAY &amp; CASH TROUGH SCHEDULE (SEGOVIA EMPIRICAL WEIGHTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Occupancy (%)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Revenue (EUR)</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Var Costs (EUR)</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Contr Margin (EUR)</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Payroll (EUR)</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Fixed OPEX (EUR)</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Debt Svc (EUR)</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>Net Op CF (EUR)</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Grant/VAT Inflow (EUR)</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>Credit Drawn (EUR)</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>Ending Cash (EUR)</t>
+        </is>
+      </c>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>Total Liquidity (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>5649.75</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>1070.21</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>4579.54</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>-5067.99</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>51682.01</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>101682.01</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>5783.4</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>1095.53</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>4687.87</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>-4959.65</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>46722.36</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>96722.36</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>9541.799999999999</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>1794.44</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>7747.36</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-1900.17</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>44822.18</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>94822.17999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>13182.75</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>2448.33</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>10734.42</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>1086.89</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>45909.08</v>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>95909.08</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>13810.5</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>2580.26</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>11230.24</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>1582.71</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>47491.78</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>97491.78</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>15734.25</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>2922.2</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>12812.05</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>3164.52</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>50656.31</v>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>100656.31</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>23101.2</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>4245.77</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>18855.43</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>9207.9</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>59864.21</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>109864.21</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>27118.8</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>4961.23</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>22157.57</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>12510.04</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="4" t="n">
+        <v>72374.25</v>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>122374.25</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>15309</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>2843.22</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>12465.78</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>2818.25</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>75192.5</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>125192.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>12555</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>2345.69</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>10209.31</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>561.78</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="4" t="n">
+        <v>75754.28</v>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>125754.28</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>8464.5</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>1591.85</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>6872.65</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>-2774.87</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>72979.39999999999</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>122979.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>12889.8</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>2380.9</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>10508.9</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>861.37</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>73840.77</v>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>123840.77</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>6277.5</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>1189.12</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>5088.38</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>-4559.15</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>69281.62</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>119281.62</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>6426</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>1217.25</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>5208.75</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>-4438.78</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>163000</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="4" t="n">
+        <v>227842.84</v>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>277842.84</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>10602</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>1993.83</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>8608.17</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>-1039.36</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>226803.48</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>276803.48</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>14647.5</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>2720.37</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>11927.13</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>2279.6</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="4" t="n">
+        <v>229083.09</v>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>279083.09</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>15345</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>2866.96</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>12478.04</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>2830.51</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>231913.6</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>281913.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>17482.5</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>3246.89</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>14235.61</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>4588.08</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>153090</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="4" t="n">
+        <v>389591.69</v>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>439591.69</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>25668</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>4717.52</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>20950.48</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>11302.95</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>400894.64</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>450894.64</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>30132</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>5512.48</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>24619.52</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>14971.99</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="4" t="n">
+        <v>415866.63</v>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>465866.63</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>17010</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>3159.13</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>13850.86</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>4203.34</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>420069.96</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>470069.96</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>13950</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>2606.32</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>11343.67</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>1696.15</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>421766.11</v>
+      </c>
+      <c r="N41" s="4" t="n">
+        <v>471766.11</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>9405</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>1768.72</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>7636.28</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>-2011.25</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>419754.86</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>469754.86</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>14322</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>2645.45</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>11676.55</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>5006.25</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>1013.25</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>3628.03</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>2029.02</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="4" t="n">
+        <v>421783.89</v>
+      </c>
+      <c r="N43" s="4" t="n">
+        <v>471783.89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement phase II landscape suites expansion and expand excel model to 8 tabs
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monte Carlo Risk" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Risk &amp; Copula" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics &amp; Runway" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase II Expansion" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4162,4 +4163,723 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="53" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PHASE II EXPANSION: LANDSCAPE HOTEL SUITES &amp; BIOLOGICAL RESERVOIR (VALUE-ADD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>1. PHASE II ALL-IN CAPEX &amp; EXECUTION BUDGET (110 M² SUITES + 200 M² POND)</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>2. INVESTMENT RETURNS &amp; CAPITAL ALLOCATION METRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>CapEx Investment Chapter</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Budget (EUR)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Technical Benchmark / Repercussion</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Return / Underwriting Parameter</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Metric Value</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Strategic Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Pure Building PEM (Foundations, Stone, Timber, Glazing, HVAC, Bath)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>161,500.00 EUR</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1,468.18 EUR/m² built (110 m²)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Stabilized Year 3 Gross Revenue</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>146,182.50 EUR</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>ADR 290 EUR net | 50% Occ (365 nights)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Contractor PEC - Pure Building (13% GG + 6% BI)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>192,185.00 EUR</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1,747.14 EUR/m² built</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Stabilized Year 3 Contribution Margin</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>114,020.52 EUR</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>78.00% contribution margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Estate Utilities &amp; Trenching Across 25 Ha (Water, Power, Bio-Sewage)</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>37,485.00 EUR</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>37,485.00 EUR PEC</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Stabilized Year 3 Incremental EBITDA</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>99,620.52 EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>68.15% EBITDA margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>5-Star FF&amp;E, High-End Textiles, Porch &amp; Exterior Hot Tub</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>41,650.00 EUR</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>41,650.00 EUR PEC (2 suites)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Stabilized Year 3 Free Cash Flow (Post-Tax)</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>75,841.41 EUR</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Clean cash flow net of 2% FF&amp;E reserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Biological Pond (200 m² EPDM, Biofilter, Zeolites, Cascade, Flora)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>38,080.00 EUR</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>38,080.00 EUR PEC (190.40 EUR/m² water)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Development Yield on Cost (EBITDA / CapEx)</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>27.67%</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Unlevered gross development yield</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL CONTRACTOR WORKS PEC (Capítulo 1 al 8)</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>309,400.00 EUR</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2,812.73 EUR/m² repercutido</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Return on Invested Capital (ROIC Y3)</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>17.38%</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+938 bps spread over 8.0% WACC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Architecture, Engineering &amp; Project Management Fees (9.0% PEM)</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>23,400.00 EUR</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Complete technical project &amp; permits</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Simple EBITDA Payback Period</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>3.99 Years</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>47.6 months recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Municipal Taxes, Urban Fees &amp; ICIO (4.5% PEM)</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>11,700.00 EUR</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Segovia rural municipality rate</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Simple Post-Tax FCF Payback Period</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>5.07 Years</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>61.2 months recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Contingency Reserve (5.0% PEC)</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>15,470.00 EUR</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Granite rock &amp; unforeseen works</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Year 5 Exit Valuation @ 8.5% Cap Rate</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>1,219,355.23 EUR</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Net gain: +859,385.23 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL ALL-IN EXPANSION CAPEX (Net of Deductible VAT)</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>359,970.00 EUR</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>179,985.00 EUR all-in per suite</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>5-Year Post-Tax IRR with Exit (8.5% Cap Rate)</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>40.29%</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>MOIC: 4.37x</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Financing Structure (Zero New Senior Debt)</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>100% Retained Cash</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Year 2 LEADER (163k) + VAT Refund (152.2k)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated Group EBITDA (Phase 1 + 2)</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>188,760.39 EUR</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>+111.76% surge vs Phase 1 baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Consolidated Debt Service Coverage (DSCR)</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>4.34x</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Expands from 2.05x to 4.34x (Zero debt add)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>3. 5-YEAR COMMERCIAL RAMP-UP &amp; CASH FLOW TRAJECTORY SCHEDULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Occupancy (%)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Nights Sold</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>ADR Net (EUR)</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Revenue (EUR)</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Contr Margin (EUR)</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>EBITDA (EUR)</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>EBIT (EUR)</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Tax 25% (EUR)</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>Net Income (EUR)</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Free Cash Flow (EUR)</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>Discounted FCF (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>37.5%</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>273.75</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>290</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>109636.88</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>85515.39</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>71115.39</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>54916.74</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>13729.19</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>41187.56</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>55193.47</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>51105.07</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>45.0%</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>328.5</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>290</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>131564.25</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>102618.47</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>88218.47</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>72019.82000000001</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>18004.96</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>54014.87</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>67582.23</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>57940.87</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>365</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>290</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>146182.5</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>114020.52</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>99620.52</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>83421.88</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>20855.47</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>62566.41</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>75841.41</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>60205.35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>365</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>295.8</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>149106.15</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>116300.94</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>101612.94</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>85414.28999999999</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>21353.57</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>64060.71</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>77277.24000000001</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>56801.08</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>365</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>301.72</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>152088.27</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>118626.95</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>103645.19</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>87446.53999999999</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>21861.64</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>65584.91</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>78741.78999999999</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>53590.34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add separate reform and resize case after the decline
The as-is three-case model is left untouched. A new overlay runs the same statements engine with a separately specified CapEx budget, external F&B and experience revenue, an incremental FTE and a movable LEADER grant.

Adds six presets (R1-R6), a value bridge that ties to the reform P&L, a CapEx by external-cover frontier, eight stress cases and a recommendation that is allowed to stay negative. Ships a 13th Excel tab, figure 7, a JSON export and eight tests.
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit Risk &amp; Copula" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics &amp; Runway" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase II Expansion" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reform Case" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,11 +28,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000000"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.00x"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,11 +71,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00BE123C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001D4ED8"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -100,14 +108,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-        <bgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,16 +179,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,12 +196,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -202,12 +216,29 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -761,425 +792,448 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Reform Case</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Separate post-decline layer: R1-R6 presets, value bridge, CapEx/cover frontier, stress tests and recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>2. THREE CASES (DO NOT CONFUSE THEM)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Revenue Y1</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>EBITDA Y1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>DSCR Y1</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Use</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Management (upside)</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>31.36%</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n">
-        <v>154548</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <v>24279.92</v>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Headline case: 31.36% mature occupancy, 1.48x the INE market average.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>INE market</t>
+          <t>Management (upside)</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>21.24%</t>
+          <t>31.36%</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>95555</v>
+        <v>154548</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>-18565.58</v>
+        <v>24279.92</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-1.46</v>
+        <v>1.34</v>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Independent benchmark: EBITDA is negative in Year 1 and does not cover debt service.</t>
+          <t>Headline case: 31.36% mature occupancy, 1.48x the INE market average.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>INE market</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>21.24%</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>95555</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>-18565.58</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Independent benchmark: EBITDA is negative in Year 1 and does not cover debt service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>Promoter (original Excel)</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>19.20%</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C24" s="8" t="n">
         <v>86275</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D24" s="8" t="n">
         <v>11297</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E24" s="9" t="n">
         <v>0.33</v>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Faithful replication of the author's original university simulator.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>3. KEY INTEGRITY CHECKS (LIVE FORMULAS)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Assets = liabilities + equity (max absolute)</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Live Model!B62:F62</t>
-        </is>
-      </c>
-      <c r="C27" s="10">
-        <f>IF(MAX(ABS('Live Model'!B62),ABS('Live Model'!C62),ABS('Live Model'!D62),ABS('Live Model'!E62),ABS('Live Model'!F62))&lt;1,"PASS","FAIL")</f>
-        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Live revenue vs. Python (Year 1)</t>
+          <t>Assets = liabilities + equity (max absolute)</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E66</t>
+          <t>Live Model!B62:F62</t>
         </is>
       </c>
       <c r="C28" s="10">
-        <f>'Live Model'!E66</f>
+        <f>IF(MAX(ABS('Live Model'!B62),ABS('Live Model'!C62),ABS('Live Model'!D62),ABS('Live Model'!E62),ABS('Live Model'!F62))&lt;1,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Live EBITDA vs. Python (Year 1)</t>
+          <t>Live revenue vs. Python (Year 1)</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E67</t>
+          <t>Live Model!E66</t>
         </is>
       </c>
       <c r="C29" s="10">
-        <f>'Live Model'!E67</f>
+        <f>'Live Model'!E66</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Live DSCR vs. Python (Year 2, binding year)</t>
+          <t>Live EBITDA vs. Python (Year 1)</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E68</t>
+          <t>Live Model!E67</t>
         </is>
       </c>
       <c r="C30" s="10">
-        <f>'Live Model'!E68</f>
+        <f>'Live Model'!E67</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Live ending cash vs. Python (Year 1)</t>
+          <t>Live DSCR vs. Python (Year 2, binding year)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E69</t>
+          <t>Live Model!E68</t>
         </is>
       </c>
       <c r="C31" s="10">
-        <f>'Live Model'!E69</f>
+        <f>'Live Model'!E68</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Live ending cash vs. Python (Year 2)</t>
+          <t>Live ending cash vs. Python (Year 1)</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E70</t>
+          <t>Live Model!E69</t>
         </is>
       </c>
       <c r="C32" s="10">
-        <f>'Live Model'!E70</f>
+        <f>'Live Model'!E69</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Live net income vs. Python (Year 1)</t>
+          <t>Live ending cash vs. Python (Year 2)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E71</t>
+          <t>Live Model!E70</t>
         </is>
       </c>
       <c r="C33" s="10">
-        <f>'Live Model'!E71</f>
+        <f>'Live Model'!E70</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>DSCR covenant (minimum of Years 1-5 &gt;= 1.25x)</t>
+          <t>Live net income vs. Python (Year 1)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Live Model!E74</t>
+          <t>Live Model!E71</t>
         </is>
       </c>
       <c r="C34" s="10">
-        <f>'Live Model'!E74</f>
+        <f>'Live Model'!E71</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Senior debt fully amortised by month 240</t>
+          <t>DSCR covenant (minimum of Years 1-5 &gt;= 1.25x)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Debt Schedule!G264</t>
+          <t>Live Model!E74</t>
         </is>
       </c>
       <c r="C35" s="10">
-        <f>IF(ABS('Debt Schedule'!G264)&lt;1,"PASS","FAIL")</f>
+        <f>'Live Model'!E74</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Sources equal uses at close (management)</t>
+          <t>Senior debt fully amortised by month 240</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Funding &amp; Audit!B27</t>
+          <t>Debt Schedule!G264</t>
         </is>
       </c>
       <c r="C36" s="10">
-        <f>IF(ABS('Funding &amp; Audit'!B27)&lt;1,"PASS","FAIL")</f>
+        <f>IF(ABS('Debt Schedule'!G264)&lt;1,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>VAT bridge within the EUR 175k limit</t>
+          <t>Sources equal uses at close (management)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Funding &amp; Audit!B23</t>
+          <t>Funding &amp; Audit!B27</t>
         </is>
       </c>
       <c r="C37" s="10">
-        <f>IF('Funding &amp; Audit'!B23&lt;=175000,"PASS","FAIL")</f>
+        <f>IF(ABS('Funding &amp; Audit'!B27)&lt;1,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t>VAT bridge within the EUR 175k limit</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Funding &amp; Audit!B23</t>
+        </is>
+      </c>
+      <c r="C38" s="10">
+        <f>IF('Funding &amp; Audit'!B23&lt;=175000,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t>Phase II phase gate</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Funding &amp; Audit!B38</t>
         </is>
       </c>
-      <c r="C38" s="10">
+      <c r="C39" s="10">
         <f>'Funding &amp; Audit'!B38</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>4. HEADLINE FINDINGS</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>- The all-in asset cost is EUR 1,050,100 (land, 550 m2 of works, kitchen, FF&amp;E, biopool, digital, fees and contingency). The cash equity plug is EUR 521,090.22, or 49.6% of CapEx, not the 30% in the business plan.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>- The EUR 367,535 facility is 35% LTV, but the binding constraint is the DSCR: the 1.25x cap supports EUR 339,144.92 (32.3% LTV). The requested loan breaches the covenant in Year 2 (1.15x).</t>
+          <t>- The all-in asset cost is EUR 1,050,100 (land, 550 m2 of works, kitchen, FF&amp;E, biopool, digital, fees and contingency). The cash equity plug is EUR 521,090.22, or 49.6% of CapEx, not the 30% in the business plan.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>- The independent INE market case (21.24%) is negative at EBITDA level in Year 1 (EUR -18,565.58) and its DSCR is -1.46x.</t>
+          <t>- The EUR 367,535 facility is 35% LTV, but the binding constraint is the DSCR: the 1.25x cap supports EUR 339,144.92 (32.3% LTV). The requested loan breaches the covenant in Year 2 (1.15x).</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>- The original promoter case (19.2%) replicates the author's university Excel (EUR 86,275 revenue / EUR 11,297 EBITDA) and is structurally insolvent at the debt service level.</t>
+          <t>- The independent INE market case (21.24%) is negative at EBITDA level in Year 1 (EUR -18,565.58) and its DSCR is -1.46x.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>- Phase II needs EUR 435,563.70 but Phase I generates EUR 183,322.64 of cash by the end of Year 2: the gate is negative by EUR 252,241.06.</t>
+          <t>- The original promoter case (19.2%) replicates the author's university Excel (EUR 86,275 revenue / EUR 11,297 EBITDA) and is structurally insolvent at the debt service level.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>- The credit-committee recommendation is DECLINE AS STRUCTURED (RESIZE REQUIRED). The covenant break-even is 32.05% occupancy or an ADR of EUR 86.64; a 10% equity IRR needs EUR 116.36.</t>
+          <t>- Phase II needs EUR 435,563.70 but Phase I generates EUR 183,322.64 of cash by the end of Year 2: the gate is negative by EUR 252,241.06.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>- The Clayton copula puts P(breach of 1.25x) at 50.7% and the worst-1% annual CFADS shortfall at EUR 62,786 against a EUR 13,824 contractual DSRA.</t>
+          <t>- The credit-committee recommendation is DECLINE AS STRUCTURED (RESIZE REQUIRED). The covenant break-even is 32.05% occupancy or an ADR of EUR 86.64; a 10% equity IRR needs EUR 116.36.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="11" t="inlineStr">
         <is>
+          <t>- The Clayton copula puts P(breach of 1.25x) at 50.7% and the worst-1% annual CFADS shortfall at EUR 62,786 against a EUR 13,824 contractual DSRA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>- The separate reform / resize layer is also negative: six external F&amp;B covers, +5% ADR and one extra FTE lift mature EBITDA to EUR 71,321 and asset value to EUR 839,075, still EUR 211,025 below the 1.05M CapEx and EUR 299,550 below total project investment. Only the aggressive eight-cover / +10% ADR corner clears 8%, and it still fails the bank test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
           <t>- The model is deliberately honest: the business does not earn its 8.5% cost of capital at the planned occupancy and ADR, and the workbook says so rather than hiding it.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>5. DISCLAIMER</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="44" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="52" ht="44" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>This is a portfolio model built from the author's own university work, public INE data and public convenio tables. It is not investment advice. The management case is an upside case; the market and promoter cases are the honest downside anchors.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="A51:F51"/>
+  <mergeCells count="10">
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A42:F42"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A43:F43"/>
   </mergeCells>
@@ -4181,6 +4235,1102 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>REFORM / RESIZE CASE - WHAT WOULD HAVE TO BE TRUE AFTER THE DECLINE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>A separate layer on top of the three as-is cases. It does not rewrite the management, INE market or promoter projections; it asks whether a revenue-led reform can create value. The answer is allowed to be no, and the conservative bank test is EV versus TOTAL project investment (CapEx + IDC + pre-opening + working capital + DSRA), not EV versus CapEx alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1. R1-R6 REFORM PRESETS (ALL SIX ARE SHOWN; NEGATIVE RESULTS ARE NOT HIDDEN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>Reform case</t>
+        </is>
+      </c>
+      <c r="C5" s="42" t="inlineStr">
+        <is>
+          <t>CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
+        <is>
+          <t>Total investment (EUR)</t>
+        </is>
+      </c>
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>Revenue Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="F5" s="42" t="inlineStr">
+        <is>
+          <t>EBITDA Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="G5" s="42" t="inlineStr">
+        <is>
+          <t>Min DSCR</t>
+        </is>
+      </c>
+      <c r="H5" s="42" t="inlineStr">
+        <is>
+          <t>EV @ exit cap (EUR)</t>
+        </is>
+      </c>
+      <c r="I5" s="42" t="inlineStr">
+        <is>
+          <t>Gap vs CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="J5" s="42" t="inlineStr">
+        <is>
+          <t>Gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="K5" s="42" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+      <c r="L5" s="42" t="inlineStr">
+        <is>
+          <t>Project IRR</t>
+        </is>
+      </c>
+      <c r="M5" s="42" t="inlineStr">
+        <is>
+          <t>Equity IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>CAPEX ONLY</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>R1 Capital-only (900k)</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="D6" s="40" t="n">
+        <v>986296.85</v>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>171720</v>
+      </c>
+      <c r="F6" s="40" t="n">
+        <v>37041.58</v>
+      </c>
+      <c r="G6" s="43" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H6" s="40" t="n">
+        <v>435783.29</v>
+      </c>
+      <c r="I6" s="40" t="n">
+        <v>-466016.71</v>
+      </c>
+      <c r="J6" s="40" t="n">
+        <v>-550513.5600000001</v>
+      </c>
+      <c r="K6" s="40" t="n">
+        <v>-450358.56</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>-0.07178</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>-0.164716</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>REVENUE REFORM</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>R2 Revenue reform (1.05M)</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>253626</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="G7" s="43" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>-211025.06</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>-299550.28</v>
+      </c>
+      <c r="K7" s="40" t="n">
+        <v>-220684.83</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>0.025297</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0.019578</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>VALUE ENGINEERED</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>R3 Revenue + value engineering (900k)</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="D8" s="40" t="n">
+        <v>986296.85</v>
+      </c>
+      <c r="E8" s="40" t="n">
+        <v>253626</v>
+      </c>
+      <c r="F8" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="G8" s="43" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="H8" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="I8" s="40" t="n">
+        <v>-62725.06</v>
+      </c>
+      <c r="J8" s="40" t="n">
+        <v>-147221.91</v>
+      </c>
+      <c r="K8" s="40" t="n">
+        <v>-96377.5</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>0.053742</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0.06250600000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>AGGRESSIVE</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>R4 Aggressive demand (1.05M)</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>282652</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>92402.75999999999</v>
+      </c>
+      <c r="G9" s="43" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>1087091.29</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>36991.29</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>-51533.93</v>
+      </c>
+      <c r="K9" s="40" t="n">
+        <v>3721.66</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.080844</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0.101638</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>RESIZE 850</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>R5 Lean scope (850k)</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>846300</v>
+      </c>
+      <c r="D10" s="40" t="n">
+        <v>929289.3100000001</v>
+      </c>
+      <c r="E10" s="40" t="n">
+        <v>253626</v>
+      </c>
+      <c r="F10" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="G10" s="43" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="H10" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="I10" s="40" t="n">
+        <v>-7225.06</v>
+      </c>
+      <c r="J10" s="40" t="n">
+        <v>-90214.37</v>
+      </c>
+      <c r="K10" s="40" t="n">
+        <v>-49105.91</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>0.066093</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.080399</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>DOWNSIDE</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>R6 Downside / stress</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>965560</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>1051789.19</v>
+      </c>
+      <c r="E11" s="40" t="n">
+        <v>187923</v>
+      </c>
+      <c r="F11" s="40" t="n">
+        <v>2670.95</v>
+      </c>
+      <c r="G11" s="43" t="n">
+        <v>-1.49</v>
+      </c>
+      <c r="H11" s="40" t="n">
+        <v>26709.5</v>
+      </c>
+      <c r="I11" s="40" t="n">
+        <v>-938850.5</v>
+      </c>
+      <c r="J11" s="40" t="n">
+        <v>-1025079.69</v>
+      </c>
+      <c r="K11" s="40" t="n">
+        <v>-906165.55</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>-0.377608</v>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2. R2 VALUE BRIDGE - MATURE EBITDA AND EV AT THE 8.5% EXIT CAP RATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>Bridge component</t>
+        </is>
+      </c>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>EBITDA impact (EUR)</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>EV impact @ 8.5% (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Base management EBITDA</t>
+        </is>
+      </c>
+      <c r="B16" s="45" t="n">
+        <v>37041.58</v>
+      </c>
+      <c r="C16" s="45" t="n">
+        <v>435783.29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>+ ADR uplift (5%)</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>7182.19</v>
+      </c>
+      <c r="C17" s="40" t="n">
+        <v>84496.35000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>+ External F&amp;B (6 covers/day)</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n">
+        <v>13697.6</v>
+      </c>
+      <c r="C18" s="40" t="n">
+        <v>161148.24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>+ Experiences</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n">
+        <v>8400</v>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>98823.53</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>+ Cost savings</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C20" s="40" t="n">
+        <v>58823.53</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Reform EBITDA and EV</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="C21" s="45" t="n">
+        <v>839074.9399999999</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Reform enterprise value @ 8.5%</t>
+        </is>
+      </c>
+      <c r="B23" s="45" t="n">
+        <v>839074.9399999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Reform CapEx</t>
+        </is>
+      </c>
+      <c r="B24" s="45" t="n">
+        <v>1050100</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Value gap vs CapEx</t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="n">
+        <v>-211025.06</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Total project investment</t>
+        </is>
+      </c>
+      <c r="B26" s="45" t="n">
+        <v>1138625.22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>3. VALUE FRONTIER - EV MINUS TOTAL INVESTMENT (EUR), BY CAPEX AND EXTERNAL COVERS</t>
+        </is>
+      </c>
+      <c r="B27" s="45" t="n">
+        <v>-299550.28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>CapEx (EUR) \ Covers/day</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="48" t="n">
+        <v>6</v>
+      </c>
+      <c r="E28" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="F28" s="48" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="45" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="B29" s="49" t="n">
+        <v>-460698.51</v>
+      </c>
+      <c r="C29" s="49" t="n">
+        <v>-544830.28</v>
+      </c>
+      <c r="D29" s="49" t="n">
+        <v>-299550.28</v>
+      </c>
+      <c r="E29" s="49" t="n">
+        <v>-245834.16</v>
+      </c>
+      <c r="F29" s="49" t="n">
+        <v>-192118.16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="45" t="n">
+        <v>950000</v>
+      </c>
+      <c r="B30" s="49" t="n">
+        <v>-357879.98</v>
+      </c>
+      <c r="C30" s="49" t="n">
+        <v>-442011.75</v>
+      </c>
+      <c r="D30" s="49" t="n">
+        <v>-196731.75</v>
+      </c>
+      <c r="E30" s="49" t="n">
+        <v>-143015.63</v>
+      </c>
+      <c r="F30" s="49" t="n">
+        <v>-89299.63</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="45" t="n">
+        <v>850000</v>
+      </c>
+      <c r="B31" s="49" t="n">
+        <v>-255162.93</v>
+      </c>
+      <c r="C31" s="49" t="n">
+        <v>-339294.7</v>
+      </c>
+      <c r="D31" s="49" t="n">
+        <v>-94014.7</v>
+      </c>
+      <c r="E31" s="49" t="n">
+        <v>-40298.58</v>
+      </c>
+      <c r="F31" s="50" t="n">
+        <v>13417.42</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="45" t="n">
+        <v>770000</v>
+      </c>
+      <c r="B32" s="49" t="n">
+        <v>-172989.81</v>
+      </c>
+      <c r="C32" s="49" t="n">
+        <v>-257121.58</v>
+      </c>
+      <c r="D32" s="49" t="n">
+        <v>-11841.58</v>
+      </c>
+      <c r="E32" s="50" t="n">
+        <v>41874.54</v>
+      </c>
+      <c r="F32" s="50" t="n">
+        <v>95590.53999999999</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="45" t="n">
+        <v>700000</v>
+      </c>
+      <c r="B33" s="49" t="n">
+        <v>-101088.63</v>
+      </c>
+      <c r="C33" s="49" t="n">
+        <v>-185220.4</v>
+      </c>
+      <c r="D33" s="50" t="n">
+        <v>60059.6</v>
+      </c>
+      <c r="E33" s="50" t="n">
+        <v>113775.72</v>
+      </c>
+      <c r="F33" s="50" t="n">
+        <v>167491.72</v>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>4. STRESS TESTS - THE REFORM UNDER DEMAND, COST, RATE AND GRANT DELAYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="51" t="inlineStr">
+        <is>
+          <t>Stress case</t>
+        </is>
+      </c>
+      <c r="B37" s="51" t="inlineStr">
+        <is>
+          <t>CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="C37" s="51" t="inlineStr">
+        <is>
+          <t>Total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="D37" s="51" t="inlineStr">
+        <is>
+          <t>EBITDA Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="E37" s="51" t="inlineStr">
+        <is>
+          <t>Min DSCR</t>
+        </is>
+      </c>
+      <c r="F37" s="51" t="inlineStr">
+        <is>
+          <t>EV (EUR)</t>
+        </is>
+      </c>
+      <c r="G37" s="51" t="inlineStr">
+        <is>
+          <t>Gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="H37" s="51" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+      <c r="I37" s="51" t="inlineStr">
+        <is>
+          <t>Project IRR</t>
+        </is>
+      </c>
+      <c r="J37" s="51" t="inlineStr">
+        <is>
+          <t>Equity IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>As-is reform (R2)</t>
+        </is>
+      </c>
+      <c r="B38" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="C38" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="D38" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E38" s="43" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F38" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G38" s="40" t="n">
+        <v>-299550.28</v>
+      </c>
+      <c r="H38" s="40" t="n">
+        <v>-220684.83</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>0.025297</v>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>0.019578</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>R2 + INE 21.24% demand</t>
+        </is>
+      </c>
+      <c r="B39" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="C39" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="D39" s="40" t="n">
+        <v>27821.26</v>
+      </c>
+      <c r="E39" s="43" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="F39" s="40" t="n">
+        <v>327308.94</v>
+      </c>
+      <c r="G39" s="40" t="n">
+        <v>-811316.28</v>
+      </c>
+      <c r="H39" s="40" t="n">
+        <v>-689417.96</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>-0.14632</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>-0.512092</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>R2 + covers -50%</t>
+        </is>
+      </c>
+      <c r="B40" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="C40" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="D40" s="40" t="n">
+        <v>50472.57</v>
+      </c>
+      <c r="E40" s="43" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F40" s="40" t="n">
+        <v>593794.9399999999</v>
+      </c>
+      <c r="G40" s="40" t="n">
+        <v>-544830.28</v>
+      </c>
+      <c r="H40" s="40" t="n">
+        <v>-441028.47</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>-0.042221</v>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>-0.102545</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>R3 + CapEx +20%</t>
+        </is>
+      </c>
+      <c r="B41" s="40" t="n">
+        <v>1032160</v>
+      </c>
+      <c r="C41" s="40" t="n">
+        <v>1120197.9</v>
+      </c>
+      <c r="D41" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E41" s="43" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F41" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G41" s="40" t="n">
+        <v>-281122.96</v>
+      </c>
+      <c r="H41" s="40" t="n">
+        <v>-206843.7</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>0.028168</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>0.024049</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>R3 + LEADER delayed to Y3</t>
+        </is>
+      </c>
+      <c r="B42" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C42" s="40" t="n">
+        <v>986296.85</v>
+      </c>
+      <c r="D42" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E42" s="43" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F42" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G42" s="40" t="n">
+        <v>-147221.91</v>
+      </c>
+      <c r="H42" s="40" t="n">
+        <v>-105254.39</v>
+      </c>
+      <c r="I42" s="7" t="n">
+        <v>0.052156</v>
+      </c>
+      <c r="J42" s="7" t="n">
+        <v>0.059813</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>R3 + rate +200 bp</t>
+        </is>
+      </c>
+      <c r="B43" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C43" s="40" t="n">
+        <v>988365</v>
+      </c>
+      <c r="D43" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E43" s="43" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F43" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G43" s="40" t="n">
+        <v>-149290.06</v>
+      </c>
+      <c r="H43" s="40" t="n">
+        <v>-98445.64999999999</v>
+      </c>
+      <c r="I43" s="7" t="n">
+        <v>0.053216</v>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0.054386</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>R3 + conservative demand</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C44" s="40" t="n">
+        <v>987831.24</v>
+      </c>
+      <c r="D44" s="40" t="n">
+        <v>33333.95</v>
+      </c>
+      <c r="E44" s="43" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F44" s="40" t="n">
+        <v>392164.12</v>
+      </c>
+      <c r="G44" s="40" t="n">
+        <v>-595667.12</v>
+      </c>
+      <c r="H44" s="40" t="n">
+        <v>-509916.1</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>-0.096315</v>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>-0.245461</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>R6 combined downside</t>
+        </is>
+      </c>
+      <c r="B45" s="40" t="n">
+        <v>965560</v>
+      </c>
+      <c r="C45" s="40" t="n">
+        <v>1051789.19</v>
+      </c>
+      <c r="D45" s="40" t="n">
+        <v>-33876</v>
+      </c>
+      <c r="E45" s="43" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="F45" s="40" t="n">
+        <v>-338760</v>
+      </c>
+      <c r="G45" s="40" t="n">
+        <v>-1390549.19</v>
+      </c>
+      <c r="H45" s="40" t="n">
+        <v>-1242114.7</v>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>5. REFORM RECOMMENDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="52" t="inlineStr">
+        <is>
+          <t>DECLINE AS STRUCTURED - ONLY THE AGGRESSIVE, UNPROVEN DEMAND CASE CLEARS THE WACC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="42" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>The realistic revenue reform (R2: six external covers/day, +5% ADR, one FTE) produces EUR 71,321 of mature EBITDA and EUR 839,075 of asset value. Against the EUR 1,050,100 CapEx that is a gap of EUR -211,025; against total project investment of EUR 1,138,625 the gap is EUR -299,550. R2 still has a project NPV of EUR -220,685 and a project IRR of 2.53%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>The 900k value-engineered case (R3) improves the NPV to EUR -96,378 and the IRR to 5.37%, but still does not clear an 8% WACC. The 850k lean case (R5) reaches EUR -49,106 of NPV and 6.61% IRR, still below the hurdle. The only positive-NPV case is R4 (eight covers/day, +10% ADR, one FTE) at EUR 3,722 of NPV and 8.08% IRR - a negligible margin and a total-investment value gap of EUR -51,534. The combined downside (R6) is deeply negative: EBITDA EUR 2,671, NPV EUR -906,166. The value frontier does show a positive corner at roughly EUR 700k of CapEx (land included) with six or more covers, but that is EUR 450k of non-land spend for an eight-room refurbishment: a scope-reduction thesis, not the current 1.05M budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Conditions attached to any further work</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>- Do not treat the 1.05M eight-room project as the base case for a reform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>- Prove external F&amp;B demand before committing construction capital: a low-cost Phase 0 pop-up/restaurant test, not a full refurbishment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>- If the family wants to proceed, cap the initial capital at the lean scope and keep the second phase behind a demand gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>- Treat the ~700k frontier corner as a different, smaller project: it only works by cutting the non-land budget to about 450k, which is not the eight-room refurbishment currently specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>- Charge the land at its opportunity value; do not describe the project as viable only because the site is already owned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>- Re-run the model with 1.25-1.5 FTE for the external covers, not one FTE, and with INE 21.24% occupancy in the downside.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A57:L57"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A54:L54"/>
+    <mergeCell ref="A51:L51"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="A58:L58"/>
+    <mergeCell ref="A56:L56"/>
+    <mergeCell ref="A55:L55"/>
+    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="A59:L59"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add occupancy bridge, net exit test and red team to the reform case
- Decompose management 31.36% vs INE 21.24% into weekend, bridge and midweek segments, with gap shares and Figure 8. - Charge 3% exit costs (4% in R6) and report net EV and net value gaps next to the gross figures. - Pin R6 to the INE occupancy anchor via ReformConfig.demand_anchor and floor the EV at zero when EBITDA is negative. - Add rate sensitivity (+0/+100/+200/+300 bp), no-LEADER stress and a solved R6 downside. - Add RED_TEAM.md / RED_TEAM_ES.md with ten attacks and responses. - Restructure both READMEs into a 60-second summary, reading map, occupancy bridge, net-exit and red-team sections. - Extend the suite to 59 tests and regenerate the 13-tab workbook and JSON artefacts.
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -230,14 +230,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -604,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1137,11 +1136,8 @@
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="n"/>
-    </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>4. HEADLINE FINDINGS</t>
         </is>
@@ -1206,31 +1202,47 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="11" t="inlineStr">
         <is>
+          <t>- The management case is 31.36% occupancy, 1.48x the INE 21.24%. It is a weekend-weighted mix, not a flat uplift: 72% weekends, 65% holiday bridges and 10% midweek reconstruct the annual target. 68% of the gap is weekend capture; the thin midweek is what the reform's external F&amp;B covers are trying to fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>- The exit is shown gross and net of 3% selling costs. R2's net value gap is EUR 324,723 against total investment; even the aggressive R4 corner fails the net test at EUR 84,147.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
           <t>- The model is deliberately honest: the business does not earn its 8.5% cost of capital at the planned occupancy and ADR, and the workbook says so rather than hiding it.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>5. DISCLAIMER</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="44" customHeight="1">
-      <c r="A52" s="12" t="inlineStr">
+    <row r="54" ht="44" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>This is a portfolio model built from the author's own university work, public INE data and public convenio tables. It is not investment advice. The management case is an upside case; the market and promoter cases are the honest downside anchors.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
+    <mergeCell ref="A54:F54"/>
     <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A51:F51"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A42:F42"/>
     <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A50:F50"/>
@@ -4245,22 +4257,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4338,15 +4351,20 @@
       </c>
       <c r="K5" s="42" t="inlineStr">
         <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="L5" s="42" t="inlineStr">
+        <is>
           <t>Project NPV (EUR)</t>
         </is>
       </c>
-      <c r="L5" s="42" t="inlineStr">
+      <c r="M5" s="42" t="inlineStr">
         <is>
           <t>Project IRR</t>
         </is>
       </c>
-      <c r="M5" s="42" t="inlineStr">
+      <c r="N5" s="42" t="inlineStr">
         <is>
           <t>Equity IRR</t>
         </is>
@@ -4388,12 +4406,15 @@
         <v>-550513.5600000001</v>
       </c>
       <c r="K6" s="40" t="n">
+        <v>-563587.0600000001</v>
+      </c>
+      <c r="L6" s="40" t="n">
         <v>-450358.56</v>
       </c>
-      <c r="L6" s="7" t="n">
+      <c r="M6" s="7" t="n">
         <v>-0.07178</v>
       </c>
-      <c r="M6" s="7" t="n">
+      <c r="N6" s="7" t="n">
         <v>-0.164716</v>
       </c>
     </row>
@@ -4433,12 +4454,15 @@
         <v>-299550.28</v>
       </c>
       <c r="K7" s="40" t="n">
+        <v>-324722.53</v>
+      </c>
+      <c r="L7" s="40" t="n">
         <v>-220684.83</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="M7" s="7" t="n">
         <v>0.025297</v>
       </c>
-      <c r="M7" s="7" t="n">
+      <c r="N7" s="7" t="n">
         <v>0.019578</v>
       </c>
     </row>
@@ -4478,12 +4502,15 @@
         <v>-147221.91</v>
       </c>
       <c r="K8" s="40" t="n">
+        <v>-172394.16</v>
+      </c>
+      <c r="L8" s="40" t="n">
         <v>-96377.5</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="M8" s="7" t="n">
         <v>0.053742</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="N8" s="7" t="n">
         <v>0.06250600000000001</v>
       </c>
     </row>
@@ -4523,12 +4550,15 @@
         <v>-51533.93</v>
       </c>
       <c r="K9" s="40" t="n">
+        <v>-84146.67</v>
+      </c>
+      <c r="L9" s="40" t="n">
         <v>3721.66</v>
       </c>
-      <c r="L9" s="7" t="n">
+      <c r="M9" s="7" t="n">
         <v>0.080844</v>
       </c>
-      <c r="M9" s="7" t="n">
+      <c r="N9" s="7" t="n">
         <v>0.101638</v>
       </c>
     </row>
@@ -4568,12 +4598,15 @@
         <v>-90214.37</v>
       </c>
       <c r="K10" s="40" t="n">
+        <v>-115386.62</v>
+      </c>
+      <c r="L10" s="40" t="n">
         <v>-49105.91</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="M10" s="7" t="n">
         <v>0.066093</v>
       </c>
-      <c r="M10" s="7" t="n">
+      <c r="N10" s="7" t="n">
         <v>0.080399</v>
       </c>
     </row>
@@ -4595,30 +4628,35 @@
         <v>1051789.19</v>
       </c>
       <c r="E11" s="40" t="n">
-        <v>187923</v>
+        <v>138035.1</v>
       </c>
       <c r="F11" s="40" t="n">
-        <v>2670.95</v>
+        <v>-33886.72</v>
       </c>
       <c r="G11" s="43" t="n">
-        <v>-1.49</v>
+        <v>-3.82</v>
       </c>
       <c r="H11" s="40" t="n">
-        <v>26709.5</v>
+        <v>0</v>
       </c>
       <c r="I11" s="40" t="n">
-        <v>-938850.5</v>
+        <v>-965560</v>
       </c>
       <c r="J11" s="40" t="n">
-        <v>-1025079.69</v>
+        <v>-1051789.19</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>-906165.55</v>
-      </c>
-      <c r="L11" s="7" t="n">
-        <v>-0.377608</v>
+        <v>-1051789.19</v>
+      </c>
+      <c r="L11" s="40" t="n">
+        <v>-1021972.82</v>
       </c>
       <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -4730,606 +4768,868 @@
     </row>
     <row r="22"/>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Reform enterprise value @ 8.5%</t>
-        </is>
-      </c>
-      <c r="B23" s="45" t="n">
-        <v>839074.9399999999</v>
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>Value test</t>
+        </is>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>Gross (EUR)</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Net of exit costs (EUR)</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Reform CapEx</t>
+          <t>Enterprise value</t>
         </is>
       </c>
       <c r="B24" s="45" t="n">
-        <v>1050100</v>
+        <v>839074.9399999999</v>
+      </c>
+      <c r="C24" s="45" t="n">
+        <v>813902.6899999999</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Value gap vs CapEx</t>
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Exit costs</t>
         </is>
       </c>
       <c r="B25" s="45" t="n">
-        <v>-211025.06</v>
+        <v>0</v>
+      </c>
+      <c r="C25" s="45" t="n">
+        <v>-25172.25</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Total project investment</t>
+          <t>Reform CapEx</t>
         </is>
       </c>
       <c r="B26" s="45" t="n">
-        <v>1138625.22</v>
+        <v>1050100</v>
+      </c>
+      <c r="C26" s="45" t="n">
+        <v>1050100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>Value gap vs CapEx</t>
+        </is>
+      </c>
+      <c r="B27" s="45" t="n">
+        <v>-211025.06</v>
+      </c>
+      <c r="C27" s="45" t="n">
+        <v>-236197.31</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Total project investment</t>
+        </is>
+      </c>
+      <c r="B28" s="45" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="C28" s="45" t="n">
+        <v>1138625.22</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Value gap vs total investment</t>
+        </is>
+      </c>
+      <c r="B29" s="45" t="n">
+        <v>-299550.28</v>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>-324722.53</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Bridge tie (must be zero)</t>
+        </is>
+      </c>
+      <c r="B30" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
           <t>3. VALUE FRONTIER - EV MINUS TOTAL INVESTMENT (EUR), BY CAPEX AND EXTERNAL COVERS</t>
         </is>
       </c>
-      <c r="B27" s="45" t="n">
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>CapEx (EUR) \ Covers/day</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="47" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" s="47" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" s="47" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="45" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="B35" s="48" t="n">
+        <v>-460698.51</v>
+      </c>
+      <c r="C35" s="48" t="n">
+        <v>-544830.28</v>
+      </c>
+      <c r="D35" s="48" t="n">
         <v>-299550.28</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="46" t="inlineStr">
-        <is>
-          <t>CapEx (EUR) \ Covers/day</t>
-        </is>
-      </c>
-      <c r="B28" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="48" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" s="48" t="n">
-        <v>6</v>
-      </c>
-      <c r="E28" s="48" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" s="48" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="45" t="n">
-        <v>1050100</v>
-      </c>
-      <c r="B29" s="49" t="n">
-        <v>-460698.51</v>
-      </c>
-      <c r="C29" s="49" t="n">
-        <v>-544830.28</v>
-      </c>
-      <c r="D29" s="49" t="n">
-        <v>-299550.28</v>
-      </c>
-      <c r="E29" s="49" t="n">
+      <c r="E35" s="48" t="n">
         <v>-245834.16</v>
       </c>
-      <c r="F29" s="49" t="n">
+      <c r="F35" s="48" t="n">
         <v>-192118.16</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="45" t="n">
+    <row r="36">
+      <c r="A36" s="45" t="n">
         <v>950000</v>
       </c>
-      <c r="B30" s="49" t="n">
+      <c r="B36" s="48" t="n">
         <v>-357879.98</v>
       </c>
-      <c r="C30" s="49" t="n">
+      <c r="C36" s="48" t="n">
         <v>-442011.75</v>
       </c>
-      <c r="D30" s="49" t="n">
+      <c r="D36" s="48" t="n">
         <v>-196731.75</v>
       </c>
-      <c r="E30" s="49" t="n">
+      <c r="E36" s="48" t="n">
         <v>-143015.63</v>
       </c>
-      <c r="F30" s="49" t="n">
+      <c r="F36" s="48" t="n">
         <v>-89299.63</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="45" t="n">
+    <row r="37">
+      <c r="A37" s="45" t="n">
         <v>850000</v>
       </c>
-      <c r="B31" s="49" t="n">
+      <c r="B37" s="48" t="n">
         <v>-255162.93</v>
       </c>
-      <c r="C31" s="49" t="n">
+      <c r="C37" s="48" t="n">
         <v>-339294.7</v>
       </c>
-      <c r="D31" s="49" t="n">
+      <c r="D37" s="48" t="n">
         <v>-94014.7</v>
       </c>
-      <c r="E31" s="49" t="n">
+      <c r="E37" s="48" t="n">
         <v>-40298.58</v>
       </c>
-      <c r="F31" s="50" t="n">
+      <c r="F37" s="49" t="n">
         <v>13417.42</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="45" t="n">
+    <row r="38">
+      <c r="A38" s="45" t="n">
         <v>770000</v>
       </c>
-      <c r="B32" s="49" t="n">
+      <c r="B38" s="48" t="n">
         <v>-172989.81</v>
       </c>
-      <c r="C32" s="49" t="n">
+      <c r="C38" s="48" t="n">
         <v>-257121.58</v>
       </c>
-      <c r="D32" s="49" t="n">
+      <c r="D38" s="48" t="n">
         <v>-11841.58</v>
       </c>
-      <c r="E32" s="50" t="n">
+      <c r="E38" s="49" t="n">
         <v>41874.54</v>
       </c>
-      <c r="F32" s="50" t="n">
+      <c r="F38" s="49" t="n">
         <v>95590.53999999999</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="45" t="n">
+    <row r="39">
+      <c r="A39" s="45" t="n">
         <v>700000</v>
       </c>
-      <c r="B33" s="49" t="n">
+      <c r="B39" s="48" t="n">
         <v>-101088.63</v>
       </c>
-      <c r="C33" s="49" t="n">
+      <c r="C39" s="48" t="n">
         <v>-185220.4</v>
       </c>
-      <c r="D33" s="50" t="n">
+      <c r="D39" s="49" t="n">
         <v>60059.6</v>
       </c>
-      <c r="E33" s="50" t="n">
+      <c r="E39" s="49" t="n">
         <v>113775.72</v>
       </c>
-      <c r="F33" s="50" t="n">
+      <c r="F39" s="49" t="n">
         <v>167491.72</v>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>4. STRESS TESTS - THE REFORM UNDER DEMAND, COST, RATE AND GRANT DELAYS</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="51" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="46" t="inlineStr">
         <is>
           <t>Stress case</t>
         </is>
       </c>
-      <c r="B37" s="51" t="inlineStr">
+      <c r="B43" s="46" t="inlineStr">
         <is>
           <t>CapEx (EUR)</t>
         </is>
       </c>
-      <c r="C37" s="51" t="inlineStr">
+      <c r="C43" s="46" t="inlineStr">
         <is>
           <t>Total inv. (EUR)</t>
         </is>
       </c>
-      <c r="D37" s="51" t="inlineStr">
+      <c r="D43" s="46" t="inlineStr">
         <is>
           <t>EBITDA Y5 (EUR)</t>
         </is>
       </c>
-      <c r="E37" s="51" t="inlineStr">
+      <c r="E43" s="46" t="inlineStr">
         <is>
           <t>Min DSCR</t>
         </is>
       </c>
-      <c r="F37" s="51" t="inlineStr">
+      <c r="F43" s="46" t="inlineStr">
         <is>
           <t>EV (EUR)</t>
         </is>
       </c>
-      <c r="G37" s="51" t="inlineStr">
+      <c r="G43" s="46" t="inlineStr">
         <is>
           <t>Gap vs total inv. (EUR)</t>
         </is>
       </c>
-      <c r="H37" s="51" t="inlineStr">
+      <c r="H43" s="46" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="I43" s="46" t="inlineStr">
         <is>
           <t>Project NPV (EUR)</t>
         </is>
       </c>
-      <c r="I37" s="51" t="inlineStr">
+      <c r="J43" s="46" t="inlineStr">
         <is>
           <t>Project IRR</t>
         </is>
       </c>
-      <c r="J37" s="51" t="inlineStr">
+      <c r="K43" s="46" t="inlineStr">
         <is>
           <t>Equity IRR</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>As-is reform (R2)</t>
-        </is>
-      </c>
-      <c r="B38" s="40" t="n">
-        <v>1050100</v>
-      </c>
-      <c r="C38" s="40" t="n">
-        <v>1138625.22</v>
-      </c>
-      <c r="D38" s="40" t="n">
-        <v>71321.37</v>
-      </c>
-      <c r="E38" s="43" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="F38" s="40" t="n">
-        <v>839074.9399999999</v>
-      </c>
-      <c r="G38" s="40" t="n">
-        <v>-299550.28</v>
-      </c>
-      <c r="H38" s="40" t="n">
-        <v>-220684.83</v>
-      </c>
-      <c r="I38" s="7" t="n">
-        <v>0.025297</v>
-      </c>
-      <c r="J38" s="7" t="n">
-        <v>0.019578</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>R2 + INE 21.24% demand</t>
-        </is>
-      </c>
-      <c r="B39" s="40" t="n">
-        <v>1050100</v>
-      </c>
-      <c r="C39" s="40" t="n">
-        <v>1138625.22</v>
-      </c>
-      <c r="D39" s="40" t="n">
-        <v>27821.26</v>
-      </c>
-      <c r="E39" s="43" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="F39" s="40" t="n">
-        <v>327308.94</v>
-      </c>
-      <c r="G39" s="40" t="n">
-        <v>-811316.28</v>
-      </c>
-      <c r="H39" s="40" t="n">
-        <v>-689417.96</v>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>-0.14632</v>
-      </c>
-      <c r="J39" s="7" t="n">
-        <v>-0.512092</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>R2 + covers -50%</t>
-        </is>
-      </c>
-      <c r="B40" s="40" t="n">
-        <v>1050100</v>
-      </c>
-      <c r="C40" s="40" t="n">
-        <v>1138625.22</v>
-      </c>
-      <c r="D40" s="40" t="n">
-        <v>50472.57</v>
-      </c>
-      <c r="E40" s="43" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F40" s="40" t="n">
-        <v>593794.9399999999</v>
-      </c>
-      <c r="G40" s="40" t="n">
-        <v>-544830.28</v>
-      </c>
-      <c r="H40" s="40" t="n">
-        <v>-441028.47</v>
-      </c>
-      <c r="I40" s="7" t="n">
-        <v>-0.042221</v>
-      </c>
-      <c r="J40" s="7" t="n">
-        <v>-0.102545</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>R3 + CapEx +20%</t>
-        </is>
-      </c>
-      <c r="B41" s="40" t="n">
-        <v>1032160</v>
-      </c>
-      <c r="C41" s="40" t="n">
-        <v>1120197.9</v>
-      </c>
-      <c r="D41" s="40" t="n">
-        <v>71321.37</v>
-      </c>
-      <c r="E41" s="43" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="F41" s="40" t="n">
-        <v>839074.9399999999</v>
-      </c>
-      <c r="G41" s="40" t="n">
-        <v>-281122.96</v>
-      </c>
-      <c r="H41" s="40" t="n">
-        <v>-206843.7</v>
-      </c>
-      <c r="I41" s="7" t="n">
-        <v>0.028168</v>
-      </c>
-      <c r="J41" s="7" t="n">
-        <v>0.024049</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>R3 + LEADER delayed to Y3</t>
-        </is>
-      </c>
-      <c r="B42" s="40" t="n">
-        <v>901800</v>
-      </c>
-      <c r="C42" s="40" t="n">
-        <v>986296.85</v>
-      </c>
-      <c r="D42" s="40" t="n">
-        <v>71321.37</v>
-      </c>
-      <c r="E42" s="43" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="F42" s="40" t="n">
-        <v>839074.9399999999</v>
-      </c>
-      <c r="G42" s="40" t="n">
-        <v>-147221.91</v>
-      </c>
-      <c r="H42" s="40" t="n">
-        <v>-105254.39</v>
-      </c>
-      <c r="I42" s="7" t="n">
-        <v>0.052156</v>
-      </c>
-      <c r="J42" s="7" t="n">
-        <v>0.059813</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>R3 + rate +200 bp</t>
-        </is>
-      </c>
-      <c r="B43" s="40" t="n">
-        <v>901800</v>
-      </c>
-      <c r="C43" s="40" t="n">
-        <v>988365</v>
-      </c>
-      <c r="D43" s="40" t="n">
-        <v>71321.37</v>
-      </c>
-      <c r="E43" s="43" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="F43" s="40" t="n">
-        <v>839074.9399999999</v>
-      </c>
-      <c r="G43" s="40" t="n">
-        <v>-149290.06</v>
-      </c>
-      <c r="H43" s="40" t="n">
-        <v>-98445.64999999999</v>
-      </c>
-      <c r="I43" s="7" t="n">
-        <v>0.053216</v>
-      </c>
-      <c r="J43" s="7" t="n">
-        <v>0.054386</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>R3 + conservative demand</t>
+          <t>As-is reform (R2)</t>
         </is>
       </c>
       <c r="B44" s="40" t="n">
-        <v>901800</v>
+        <v>1050100</v>
       </c>
       <c r="C44" s="40" t="n">
-        <v>987831.24</v>
+        <v>1138625.22</v>
       </c>
       <c r="D44" s="40" t="n">
-        <v>33333.95</v>
+        <v>71321.37</v>
       </c>
       <c r="E44" s="43" t="n">
-        <v>0.12</v>
+        <v>2.13</v>
       </c>
       <c r="F44" s="40" t="n">
-        <v>392164.12</v>
+        <v>839074.9399999999</v>
       </c>
       <c r="G44" s="40" t="n">
-        <v>-595667.12</v>
+        <v>-299550.28</v>
       </c>
       <c r="H44" s="40" t="n">
-        <v>-509916.1</v>
-      </c>
-      <c r="I44" s="7" t="n">
-        <v>-0.096315</v>
+        <v>-324722.53</v>
+      </c>
+      <c r="I44" s="40" t="n">
+        <v>-220684.83</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>-0.245461</v>
+        <v>0.025297</v>
+      </c>
+      <c r="K44" s="7" t="n">
+        <v>0.019578</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
+          <t>R2 + INE 21.24% demand</t>
+        </is>
+      </c>
+      <c r="B45" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="C45" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="D45" s="40" t="n">
+        <v>27821.26</v>
+      </c>
+      <c r="E45" s="43" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="F45" s="40" t="n">
+        <v>327308.94</v>
+      </c>
+      <c r="G45" s="40" t="n">
+        <v>-811316.28</v>
+      </c>
+      <c r="H45" s="40" t="n">
+        <v>-821135.55</v>
+      </c>
+      <c r="I45" s="40" t="n">
+        <v>-689417.96</v>
+      </c>
+      <c r="J45" s="7" t="n">
+        <v>-0.14632</v>
+      </c>
+      <c r="K45" s="7" t="n">
+        <v>-0.512092</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>R2 + covers -50%</t>
+        </is>
+      </c>
+      <c r="B46" s="40" t="n">
+        <v>1050100</v>
+      </c>
+      <c r="C46" s="40" t="n">
+        <v>1138625.22</v>
+      </c>
+      <c r="D46" s="40" t="n">
+        <v>50472.57</v>
+      </c>
+      <c r="E46" s="43" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F46" s="40" t="n">
+        <v>593794.9399999999</v>
+      </c>
+      <c r="G46" s="40" t="n">
+        <v>-544830.28</v>
+      </c>
+      <c r="H46" s="40" t="n">
+        <v>-562644.13</v>
+      </c>
+      <c r="I46" s="40" t="n">
+        <v>-441028.47</v>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>-0.042221</v>
+      </c>
+      <c r="K46" s="7" t="n">
+        <v>-0.102545</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>R3 + CapEx +20%</t>
+        </is>
+      </c>
+      <c r="B47" s="40" t="n">
+        <v>1032160</v>
+      </c>
+      <c r="C47" s="40" t="n">
+        <v>1120197.9</v>
+      </c>
+      <c r="D47" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E47" s="43" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F47" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G47" s="40" t="n">
+        <v>-281122.96</v>
+      </c>
+      <c r="H47" s="40" t="n">
+        <v>-306295.21</v>
+      </c>
+      <c r="I47" s="40" t="n">
+        <v>-206843.7</v>
+      </c>
+      <c r="J47" s="7" t="n">
+        <v>0.028168</v>
+      </c>
+      <c r="K47" s="7" t="n">
+        <v>0.024049</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>R3 + LEADER delayed to Y3</t>
+        </is>
+      </c>
+      <c r="B48" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C48" s="40" t="n">
+        <v>986296.85</v>
+      </c>
+      <c r="D48" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E48" s="43" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F48" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G48" s="40" t="n">
+        <v>-147221.91</v>
+      </c>
+      <c r="H48" s="40" t="n">
+        <v>-172394.16</v>
+      </c>
+      <c r="I48" s="40" t="n">
+        <v>-105254.39</v>
+      </c>
+      <c r="J48" s="7" t="n">
+        <v>0.052156</v>
+      </c>
+      <c r="K48" s="7" t="n">
+        <v>0.059813</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>R3 + no LEADER grant</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C49" s="40" t="n">
+        <v>986296.85</v>
+      </c>
+      <c r="D49" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E49" s="43" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F49" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G49" s="40" t="n">
+        <v>-147221.91</v>
+      </c>
+      <c r="H49" s="40" t="n">
+        <v>-172394.16</v>
+      </c>
+      <c r="I49" s="40" t="n">
+        <v>-216215.47</v>
+      </c>
+      <c r="J49" s="7" t="n">
+        <v>0.022505</v>
+      </c>
+      <c r="K49" s="7" t="n">
+        <v>0.016396</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>R3 + rate +200 bp</t>
+        </is>
+      </c>
+      <c r="B50" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C50" s="40" t="n">
+        <v>988365</v>
+      </c>
+      <c r="D50" s="40" t="n">
+        <v>71321.37</v>
+      </c>
+      <c r="E50" s="43" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F50" s="40" t="n">
+        <v>839074.9399999999</v>
+      </c>
+      <c r="G50" s="40" t="n">
+        <v>-149290.06</v>
+      </c>
+      <c r="H50" s="40" t="n">
+        <v>-174462.31</v>
+      </c>
+      <c r="I50" s="40" t="n">
+        <v>-98445.64999999999</v>
+      </c>
+      <c r="J50" s="7" t="n">
+        <v>0.053216</v>
+      </c>
+      <c r="K50" s="7" t="n">
+        <v>0.054386</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>R3 + conservative demand</t>
+        </is>
+      </c>
+      <c r="B51" s="40" t="n">
+        <v>901800</v>
+      </c>
+      <c r="C51" s="40" t="n">
+        <v>987831.24</v>
+      </c>
+      <c r="D51" s="40" t="n">
+        <v>33333.95</v>
+      </c>
+      <c r="E51" s="43" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F51" s="40" t="n">
+        <v>392164.12</v>
+      </c>
+      <c r="G51" s="40" t="n">
+        <v>-595667.12</v>
+      </c>
+      <c r="H51" s="40" t="n">
+        <v>-607432.04</v>
+      </c>
+      <c r="I51" s="40" t="n">
+        <v>-509916.1</v>
+      </c>
+      <c r="J51" s="7" t="n">
+        <v>-0.096315</v>
+      </c>
+      <c r="K51" s="7" t="n">
+        <v>-0.245461</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
           <t>R6 combined downside</t>
         </is>
       </c>
-      <c r="B45" s="40" t="n">
+      <c r="B52" s="40" t="n">
         <v>965560</v>
       </c>
-      <c r="C45" s="40" t="n">
+      <c r="C52" s="40" t="n">
         <v>1051789.19</v>
       </c>
-      <c r="D45" s="40" t="n">
-        <v>-33876</v>
-      </c>
-      <c r="E45" s="43" t="n">
+      <c r="D52" s="40" t="n">
+        <v>-33886.72</v>
+      </c>
+      <c r="E52" s="43" t="n">
         <v>-3.82</v>
       </c>
-      <c r="F45" s="40" t="n">
-        <v>-338760</v>
-      </c>
-      <c r="G45" s="40" t="n">
-        <v>-1390549.19</v>
-      </c>
-      <c r="H45" s="40" t="n">
-        <v>-1242114.7</v>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="F52" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="40" t="n">
+        <v>-1051789.19</v>
+      </c>
+      <c r="H52" s="40" t="n">
+        <v>-1051789.19</v>
+      </c>
+      <c r="I52" s="40" t="n">
+        <v>-1021972.82</v>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="K52" s="6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>5. REFORM RECOMMENDATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="52" t="inlineStr">
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>5. RATE SENSITIVITY - R2 REFORM AT +0 / +100 / +200 / +300 BP</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="46" t="inlineStr">
+        <is>
+          <t>Rate shock (bp)</t>
+        </is>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>Interest rate</t>
+        </is>
+      </c>
+      <c r="C56" s="46" t="inlineStr">
+        <is>
+          <t>Min DSCR</t>
+        </is>
+      </c>
+      <c r="D56" s="46" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>Gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="F56" s="46" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C57" s="43" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="D57" s="40" t="n">
+        <v>-220684.83</v>
+      </c>
+      <c r="E57" s="40" t="n">
+        <v>-299550.28</v>
+      </c>
+      <c r="F57" s="40" t="n">
+        <v>-324722.53</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="50" t="n">
+        <v>100</v>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C58" s="43" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="D58" s="40" t="n">
+        <v>-221862.57</v>
+      </c>
+      <c r="E58" s="40" t="n">
+        <v>-300728.02</v>
+      </c>
+      <c r="F58" s="40" t="n">
+        <v>-325900.27</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="50" t="n">
+        <v>200</v>
+      </c>
+      <c r="B59" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C59" s="43" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D59" s="40" t="n">
+        <v>-223093.76</v>
+      </c>
+      <c r="E59" s="40" t="n">
+        <v>-301959.21</v>
+      </c>
+      <c r="F59" s="40" t="n">
+        <v>-327131.46</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="50" t="n">
+        <v>300</v>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C60" s="43" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D60" s="40" t="n">
+        <v>-224375.72</v>
+      </c>
+      <c r="E60" s="40" t="n">
+        <v>-303241.17</v>
+      </c>
+      <c r="F60" s="40" t="n">
+        <v>-328413.42</v>
+      </c>
+    </row>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>6. REFORM RECOMMENDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="51" t="inlineStr">
         <is>
           <t>DECLINE AS STRUCTURED - ONLY THE AGGRESSIVE, UNPROVEN DEMAND CASE CLEARS THE WACC</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="42" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>The realistic revenue reform (R2: six external covers/day, +5% ADR, one FTE) produces EUR 71,321 of mature EBITDA and EUR 839,075 of asset value. Against the EUR 1,050,100 CapEx that is a gap of EUR -211,025; against total project investment of EUR 1,138,625 the gap is EUR -299,550. R2 still has a project NPV of EUR -220,685 and a project IRR of 2.53%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="42" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>The 900k value-engineered case (R3) improves the NPV to EUR -96,378 and the IRR to 5.37%, but still does not clear an 8% WACC. The 850k lean case (R5) reaches EUR -49,106 of NPV and 6.61% IRR, still below the hurdle. The only positive-NPV case is R4 (eight covers/day, +10% ADR, one FTE) at EUR 3,722 of NPV and 8.08% IRR - a negligible margin and a total-investment value gap of EUR -51,534. The combined downside (R6) is deeply negative: EBITDA EUR 2,671, NPV EUR -906,166. The value frontier does show a positive corner at roughly EUR 700k of CapEx (land included) with six or more covers, but that is EUR 450k of non-land spend for an eight-room refurbishment: a scope-reduction thesis, not the current 1.05M budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52"/>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="65" ht="46" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>The realistic revenue reform (R2: six external covers/day, +5% ADR, one FTE) produces EUR 71,321 of mature EBITDA and EUR 839,075 of asset value. Against the EUR 1,050,100 CapEx that is a gap of EUR -211,025; against total project investment of EUR 1,138,625 the gap is EUR -299,550. After 3.0% exit costs the net gap is EUR -324,723. R2 still has a project NPV of EUR -220,685 and a project IRR of 2.53%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="56" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>The 900k value-engineered case (R3) improves the NPV to EUR -96,378 and the IRR to 5.37%, but still does not clear an 8% WACC. The 850k lean case (R5) reaches EUR -49,106 of NPV and 6.61% IRR, still below the hurdle. The only positive-NPV case is R4 (eight covers/day, +10% ADR, one FTE) at EUR 3,722 of NPV and 8.08% IRR - a negligible margin and a total-investment value gap of EUR -51,534. After 3.0% exit costs the net gap is EUR -84,147, so even the boundary case fails the net test. The combined downside (R6) is deeply negative: EBITDA EUR -33,887, NPV EUR -1,021,973. The value frontier does show a positive corner at roughly EUR 700k of CapEx (land included) with six or more covers, but that is EUR 450k of non-land spend for an eight-room refurbishment: a scope-reduction thesis, not the current 1.05M budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67"/>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Conditions attached to any further work</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>- Do not treat the 1.05M eight-room project as the base case for a reform.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>- Prove external F&amp;B demand before committing construction capital: a low-cost Phase 0 pop-up/restaurant test, not a full refurbishment.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
+    <row r="71" ht="28" customHeight="1">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t>- If the family wants to proceed, cap the initial capital at the lean scope and keep the second phase behind a demand gate.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="72" ht="28" customHeight="1">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>- Treat the ~700k frontier corner as a different, smaller project: it only works by cutting the non-land budget to about 450k, which is not the eight-room refurbishment currently specified.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="11" t="inlineStr">
         <is>
           <t>- Charge the land at its opportunity value; do not describe the project as viable only because the site is already owned.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+    <row r="74" ht="28" customHeight="1">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>- Price the exit net of selling costs. The gross cap-rate value flatters every case; the boundary case fails once 3% exit costs are deducted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t>- Re-run the model with 1.25-1.5 FTE for the external covers, not one FTE, and with INE 21.24% occupancy in the downside.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A57:L57"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A54:L54"/>
-    <mergeCell ref="A51:L51"/>
-    <mergeCell ref="A49:L49"/>
-    <mergeCell ref="A58:L58"/>
-    <mergeCell ref="A56:L56"/>
-    <mergeCell ref="A55:L55"/>
-    <mergeCell ref="A50:L50"/>
-    <mergeCell ref="A59:L59"/>
+  <mergeCells count="11">
+    <mergeCell ref="A70:N70"/>
+    <mergeCell ref="A69:N69"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A72:N72"/>
+    <mergeCell ref="A64:N64"/>
+    <mergeCell ref="A65:N65"/>
+    <mergeCell ref="A73:N73"/>
+    <mergeCell ref="A71:N71"/>
+    <mergeCell ref="A75:N75"/>
+    <mergeCell ref="A66:N66"/>
+    <mergeCell ref="A74:N74"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add R7 premium cabins as a separate reform preset
- Add CABIN_PRESETS (base, stretch, downside) with cabin unit mix,
  occupancy ramp, external service days and extra fixed OPEX.
- Extend the statements engine with a cabins calibration mode and
  route R7 through the existing three-statement overlay.
- Add run_cabin_presets, cabin_cost_ladder and cabin_recommendation;
  the ladder verdict uses the net total-investment test, not gross CapEx.
- Export sections 7-9 to the Excel Reform Case tab and the JSON.
- Add six R7 tests (65 total), five red-team attacks (15 total) and
  the R7 limitation to both READMEs.
- Refresh the benchmarks note with the engine reconciliation.
- Regenerate the Excel workbook and reform_analysis.json.
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +72,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00BE123C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F766E"/>
       <sz val="12"/>
     </font>
     <font>
@@ -157,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,11 +185,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -216,10 +222,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -238,6 +244,8 @@
     <xf numFmtId="3" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -799,7 +807,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Separate post-decline layer: R1-R6 presets, value bridge, CapEx/cover frontier, stress tests and recommendation.</t>
+          <t>Separate post-decline layer: R1-R6 presets, value bridge, CapEx/cover frontier, stress tests, R7 premium cabins and recommendation.</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4269,7 +4277,7 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
@@ -5617,19 +5625,519 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>7. R7 PREMIUM CABINS - A DIFFERENT PRODUCT, SAME 9.5% CAP-RATE HURDLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="42" customHeight="1">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>R7 replaces the eight-room hotel with six two-bedroom cabins plus the main house. The base case is deliberately the good edge of the band: 6 cabins at 110k all-in, 200 EUR ADR, 50% stabilised occupancy, ten external covers and 45k of experiences. At 120k per cabin the same demand fails the bank-facing net total-investment test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="42" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B79" s="42" t="inlineStr">
+        <is>
+          <t>Cabins</t>
+        </is>
+      </c>
+      <c r="C79" s="42" t="inlineStr">
+        <is>
+          <t>ADR (EUR)</t>
+        </is>
+      </c>
+      <c r="D79" s="42" t="inlineStr">
+        <is>
+          <t>Occupancy</t>
+        </is>
+      </c>
+      <c r="E79" s="42" t="inlineStr">
+        <is>
+          <t>Cost / cabin (EUR)</t>
+        </is>
+      </c>
+      <c r="F79" s="42" t="inlineStr">
+        <is>
+          <t>CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="G79" s="42" t="inlineStr">
+        <is>
+          <t>Total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="H79" s="42" t="inlineStr">
+        <is>
+          <t>EBITDA Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="I79" s="42" t="inlineStr">
+        <is>
+          <t>Min DSCR</t>
+        </is>
+      </c>
+      <c r="J79" s="42" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="K79" s="42" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+      <c r="L79" s="42" t="inlineStr">
+        <is>
+          <t>Project IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>CABINS BASE</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" s="40" t="n">
+        <v>200</v>
+      </c>
+      <c r="D80" s="52" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E80" s="40" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F80" s="40" t="n">
+        <v>1441600</v>
+      </c>
+      <c r="G80" s="40" t="n">
+        <v>1540760.04</v>
+      </c>
+      <c r="H80" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="I80" s="43" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J80" s="40" t="n">
+        <v>49146.54</v>
+      </c>
+      <c r="K80" s="40" t="n">
+        <v>76416.23</v>
+      </c>
+      <c r="L80" s="7" t="n">
+        <v>0.092088</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>CABINS STRETCH</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C81" s="40" t="n">
+        <v>230</v>
+      </c>
+      <c r="D81" s="52" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E81" s="40" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F81" s="40" t="n">
+        <v>1708000</v>
+      </c>
+      <c r="G81" s="40" t="n">
+        <v>1814396.63</v>
+      </c>
+      <c r="H81" s="40" t="n">
+        <v>227340.1</v>
+      </c>
+      <c r="I81" s="43" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J81" s="40" t="n">
+        <v>506865.44</v>
+      </c>
+      <c r="K81" s="40" t="n">
+        <v>509113.02</v>
+      </c>
+      <c r="L81" s="7" t="n">
+        <v>0.143285</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>CABINS DOWNSIDE</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="D82" s="52" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E82" s="40" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F82" s="40" t="n">
+        <v>1541500</v>
+      </c>
+      <c r="G82" s="40" t="n">
+        <v>1643374.02</v>
+      </c>
+      <c r="H82" s="40" t="n">
+        <v>71597.62</v>
+      </c>
+      <c r="I82" s="43" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J82" s="40" t="n">
+        <v>-988767.2</v>
+      </c>
+      <c r="K82" s="40" t="n">
+        <v>-878138.02</v>
+      </c>
+      <c r="L82" s="7" t="n">
+        <v>-0.092334</v>
+      </c>
+    </row>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>8. R7 COST CORRIDOR - SIX CABINS, 200 EUR ADR, 50% OCCUPANCY (PASS = NET TOTAL-INVESTMENT TEST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="42" t="inlineStr">
+        <is>
+          <t>Cost / cabin (EUR)</t>
+        </is>
+      </c>
+      <c r="B86" s="42" t="inlineStr">
+        <is>
+          <t>CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="C86" s="42" t="inlineStr">
+        <is>
+          <t>Total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="D86" s="42" t="inlineStr">
+        <is>
+          <t>EBITDA Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="E86" s="42" t="inlineStr">
+        <is>
+          <t>EV (EUR)</t>
+        </is>
+      </c>
+      <c r="F86" s="42" t="inlineStr">
+        <is>
+          <t>Gap vs CapEx (EUR)</t>
+        </is>
+      </c>
+      <c r="G86" s="42" t="inlineStr">
+        <is>
+          <t>Gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="H86" s="42" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="I86" s="42" t="inlineStr">
+        <is>
+          <t>Min DSCR</t>
+        </is>
+      </c>
+      <c r="J86" s="42" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="45" t="n">
+        <v>110000</v>
+      </c>
+      <c r="B87" s="40" t="n">
+        <v>1441600</v>
+      </c>
+      <c r="C87" s="40" t="n">
+        <v>1540760.04</v>
+      </c>
+      <c r="D87" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="E87" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F87" s="40" t="n">
+        <v>197478.95</v>
+      </c>
+      <c r="G87" s="40" t="n">
+        <v>98318.91</v>
+      </c>
+      <c r="H87" s="49" t="n">
+        <v>49146.54</v>
+      </c>
+      <c r="I87" s="43" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J87" s="40" t="n">
+        <v>76416.23</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="45" t="n">
+        <v>120000</v>
+      </c>
+      <c r="B88" s="40" t="n">
+        <v>1508200</v>
+      </c>
+      <c r="C88" s="40" t="n">
+        <v>1609169.17</v>
+      </c>
+      <c r="D88" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="E88" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F88" s="40" t="n">
+        <v>130878.95</v>
+      </c>
+      <c r="G88" s="40" t="n">
+        <v>29909.78</v>
+      </c>
+      <c r="H88" s="48" t="n">
+        <v>-19262.59</v>
+      </c>
+      <c r="I88" s="43" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J88" s="40" t="n">
+        <v>10001.46</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="45" t="n">
+        <v>130000</v>
+      </c>
+      <c r="B89" s="40" t="n">
+        <v>1574800</v>
+      </c>
+      <c r="C89" s="40" t="n">
+        <v>1677578.94</v>
+      </c>
+      <c r="D89" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="E89" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F89" s="40" t="n">
+        <v>64278.95</v>
+      </c>
+      <c r="G89" s="40" t="n">
+        <v>-38499.99</v>
+      </c>
+      <c r="H89" s="48" t="n">
+        <v>-87672.36</v>
+      </c>
+      <c r="I89" s="43" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J89" s="40" t="n">
+        <v>-56413.95</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="45" t="n">
+        <v>150000</v>
+      </c>
+      <c r="B90" s="40" t="n">
+        <v>1708000</v>
+      </c>
+      <c r="C90" s="40" t="n">
+        <v>1814396.63</v>
+      </c>
+      <c r="D90" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="E90" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F90" s="40" t="n">
+        <v>-68921.05</v>
+      </c>
+      <c r="G90" s="40" t="n">
+        <v>-175317.68</v>
+      </c>
+      <c r="H90" s="48" t="n">
+        <v>-224490.05</v>
+      </c>
+      <c r="I90" s="43" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J90" s="40" t="n">
+        <v>-189242.92</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="45" t="n">
+        <v>180000</v>
+      </c>
+      <c r="B91" s="40" t="n">
+        <v>1907800</v>
+      </c>
+      <c r="C91" s="40" t="n">
+        <v>2019624.19</v>
+      </c>
+      <c r="D91" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="E91" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F91" s="40" t="n">
+        <v>-268721.05</v>
+      </c>
+      <c r="G91" s="40" t="n">
+        <v>-380545.24</v>
+      </c>
+      <c r="H91" s="48" t="n">
+        <v>-429717.61</v>
+      </c>
+      <c r="I91" s="43" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J91" s="40" t="n">
+        <v>-388487.41</v>
+      </c>
+    </row>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>9. R7 CABIN RECOMMENDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="53" t="inlineStr">
+        <is>
+          <t>CONDITIONAL PROCEED TO PHASE 0 - PREMIUM CABINS PASS ON PAPER, BUT ONLY AT 110K PER CABIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="46" customHeight="1">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>The base cabin case (six two-bedroom cabins, 200 EUR ADR, 50% occupancy, ten external covers, 45k of experiences) produces EUR 155,712 of mature EBITDA and EUR 1,639,079 of enterprise value at a 9.5% cap rate. Against total investment of EUR 1,540,760 that is a net gap of EUR +49,147 after 3.0% selling costs: it passes, but by roughly 3.2% of the capital at risk. The project NPV is EUR +76,416, the project IRR 9.21% and the minimum DSCR 1.41x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="56" customHeight="1">
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t>The corridor is narrow. At 120k per cabin the same demand fails the net total-investment test, and at 150k it only works if the ADR moves to 230 EUR and occupancy to 55% (the stretch case: EBITDA EUR 227,340, net gap EUR +506,865). The 180k ultra-luxury unit fails with the demand this market pays. The downside (five cabins, 190 EUR, 45% occupancy) produces EBITDA EUR 71,598, a minimum DSCR of 0.79x and a net gap of EUR -988,767: it is a demand failure, not a construction-cost problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98"/>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>R7 conditions attached to any further work</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>- Run the Phase 0 demand test before committing construction capital: two cabins plus the house for one season, or a restaurant/experience pop-up. The gates are 45% occupancy, 190 EUR realised ADR, eight external covers a day and 25k of experiences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="11" t="inlineStr">
+        <is>
+          <t>- Keep the all-in cabin cost at or below 110k. At 120k the same demand band fails the net total-investment test; at 130k or more the gap is negative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1">
+      <c r="A102" s="11" t="inlineStr">
+        <is>
+          <t>- Do not budget the 180k ultra-luxury unit. It only works at 250 EUR ADR or more, which the Segovia comparables do not support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="11" t="inlineStr">
+        <is>
+          <t>- Treat the 45k of agronomic experiences as an operating programme with a host, a calendar and marketing, not as passive income.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="28" customHeight="1">
+      <c r="A104" s="11" t="inlineStr">
+        <is>
+          <t>- Charge the land at its 250k opportunity value; the case does not pass by treating the site as free.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="20">
+    <mergeCell ref="A77:N77"/>
+    <mergeCell ref="A64:N64"/>
+    <mergeCell ref="A73:N73"/>
+    <mergeCell ref="A103:N103"/>
     <mergeCell ref="A70:N70"/>
     <mergeCell ref="A69:N69"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A72:N72"/>
-    <mergeCell ref="A64:N64"/>
     <mergeCell ref="A65:N65"/>
-    <mergeCell ref="A73:N73"/>
-    <mergeCell ref="A71:N71"/>
     <mergeCell ref="A75:N75"/>
     <mergeCell ref="A66:N66"/>
     <mergeCell ref="A74:N74"/>
+    <mergeCell ref="A101:N101"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A104:N104"/>
+    <mergeCell ref="A95:N95"/>
+    <mergeCell ref="A71:N71"/>
+    <mergeCell ref="A97:N97"/>
+    <mergeCell ref="A100:N100"/>
+    <mergeCell ref="A96:N96"/>
+    <mergeCell ref="A72:N72"/>
+    <mergeCell ref="A102:N102"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add R7 robustness tests and model governance pack
Add a valuation cross-check (development yield vs exit cap, break-even cap, no-compression case and exit-multiple table), an asymmetric real cost-inflation stress and a downside distress playbook to the R7 layer. Export all three to the Reform Case tab and to data/reform_analysis.json.

Add MODEL_GOVERNANCE.md and MODEL_GOVERNANCE_ES.md: model map, calculation flow, conventions, assumption log, audit-exception disposition and change control. Refresh README, red-team memos and the R7 benchmarks note to 68 tests, seventeen attacks and the narrower 30bp/2% margin.
</commit_message>
<xml_diff>
--- a/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
+++ b/data/La_Dehesa_del_Castrillo_Financial_Model.xlsx
@@ -28,12 +28,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.00x"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0x"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +82,12 @@
       <b val="1"/>
       <color rgb="000F766E"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00BE123C"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -163,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,16 +194,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="9" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -222,10 +231,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -246,6 +255,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4265,13 +4282,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N104"/>
+  <dimension ref="A1:N150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
@@ -6116,15 +6133,609 @@
         </is>
       </c>
     </row>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>10. R7 VALUATION CROSS-CHECK - DEVELOPMENT YIELD vs EXIT CAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="40" customHeight="1">
+      <c r="A108" s="12" t="inlineStr">
+        <is>
+          <t>The positive gap is a development spread: the asset is built at a 10.1% yield on cost and sold at a 9.5% cap. The break-even exit cap is only 30bp above the assumption; at no compression the net gap is just the exit costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>Development yield on cost</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="n">
+        <v>0.1011</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Exit cap rate</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="n">
+        <v>0.095</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>Break-even exit cap (net of costs)</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="n">
+        <v>0.098</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>Cap-rate headroom (bp)</t>
+        </is>
+      </c>
+      <c r="B112" s="54" t="n">
+        <v>30.3</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>No-compression net gap (EUR)</t>
+        </is>
+      </c>
+      <c r="B113" s="40" t="n">
+        <v>-46222.8</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>Break-even EBITDA, net (EUR)</t>
+        </is>
+      </c>
+      <c r="B114" s="40" t="n">
+        <v>150899.18</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>EBITDA headroom (EUR)</t>
+        </is>
+      </c>
+      <c r="B115" s="40" t="n">
+        <v>4813.32</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>Implied exit multiple</t>
+        </is>
+      </c>
+      <c r="B116" s="43" t="n">
+        <v>10.53</v>
+      </c>
+    </row>
+    <row r="117"/>
+    <row r="118">
+      <c r="A118" s="42" t="inlineStr">
+        <is>
+          <t>Exit multiple</t>
+        </is>
+      </c>
+      <c r="B118" s="42" t="inlineStr">
+        <is>
+          <t>EV (EUR)</t>
+        </is>
+      </c>
+      <c r="C118" s="42" t="inlineStr">
+        <is>
+          <t>Net exit value (EUR)</t>
+        </is>
+      </c>
+      <c r="D118" s="42" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="B119" s="40" t="n">
+        <v>1401412.5</v>
+      </c>
+      <c r="C119" s="40" t="n">
+        <v>1359370.12</v>
+      </c>
+      <c r="D119" s="48" t="n">
+        <v>-181389.92</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="55" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="B120" s="40" t="n">
+        <v>1634981.25</v>
+      </c>
+      <c r="C120" s="40" t="n">
+        <v>1585931.81</v>
+      </c>
+      <c r="D120" s="49" t="n">
+        <v>45171.77</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="B121" s="40" t="n">
+        <v>1868550</v>
+      </c>
+      <c r="C121" s="40" t="n">
+        <v>1812493.5</v>
+      </c>
+      <c r="D121" s="49" t="n">
+        <v>271733.46</v>
+      </c>
+    </row>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>11. R7 COST-INFLATION STRESS - REAL COST GROWTH, FLAT REAL PRICES</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="42" t="inlineStr">
+        <is>
+          <t>Cost inflation / yr</t>
+        </is>
+      </c>
+      <c r="B125" s="42" t="inlineStr">
+        <is>
+          <t>EBITDA Y5 (EUR)</t>
+        </is>
+      </c>
+      <c r="C125" s="42" t="inlineStr">
+        <is>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+      <c r="D125" s="42" t="inlineStr">
+        <is>
+          <t>DSCR Y5</t>
+        </is>
+      </c>
+      <c r="E125" s="42" t="inlineStr">
+        <is>
+          <t>EV (EUR)</t>
+        </is>
+      </c>
+      <c r="F125" s="42" t="inlineStr">
+        <is>
+          <t>Net gap vs total inv. (EUR)</t>
+        </is>
+      </c>
+      <c r="G125" s="42" t="inlineStr">
+        <is>
+          <t>Project NPV (EUR)</t>
+        </is>
+      </c>
+      <c r="H125" s="42" t="inlineStr">
+        <is>
+          <t>Project IRR</t>
+        </is>
+      </c>
+      <c r="I125" s="42" t="inlineStr">
+        <is>
+          <t>Net test</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="B126" s="40" t="n">
+        <v>155712.5</v>
+      </c>
+      <c r="C126" s="56" t="n">
+        <v>0.2717</v>
+      </c>
+      <c r="D126" s="43" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E126" s="40" t="n">
+        <v>1639078.95</v>
+      </c>
+      <c r="F126" s="40" t="n">
+        <v>49146.54</v>
+      </c>
+      <c r="G126" s="40" t="n">
+        <v>76416.23</v>
+      </c>
+      <c r="H126" s="7" t="n">
+        <v>0.092088</v>
+      </c>
+      <c r="I126" s="57" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="56" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="B127" s="40" t="n">
+        <v>136911.79</v>
+      </c>
+      <c r="C127" s="56" t="n">
+        <v>0.2389</v>
+      </c>
+      <c r="D127" s="43" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E127" s="40" t="n">
+        <v>1441176.74</v>
+      </c>
+      <c r="F127" s="40" t="n">
+        <v>-142818.6</v>
+      </c>
+      <c r="G127" s="40" t="n">
+        <v>-83984.03</v>
+      </c>
+      <c r="H127" s="7" t="n">
+        <v>0.06605999999999999</v>
+      </c>
+      <c r="I127" s="58" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="56" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="B128" s="40" t="n">
+        <v>132035.38</v>
+      </c>
+      <c r="C128" s="56" t="n">
+        <v>0.2304</v>
+      </c>
+      <c r="D128" s="43" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="E128" s="40" t="n">
+        <v>1389846.11</v>
+      </c>
+      <c r="F128" s="40" t="n">
+        <v>-192609.31</v>
+      </c>
+      <c r="G128" s="40" t="n">
+        <v>-125501.41</v>
+      </c>
+      <c r="H128" s="7" t="n">
+        <v>0.058889</v>
+      </c>
+      <c r="I128" s="58" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="56" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="B129" s="40" t="n">
+        <v>127087.08</v>
+      </c>
+      <c r="C129" s="56" t="n">
+        <v>0.2218</v>
+      </c>
+      <c r="D129" s="43" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="E129" s="40" t="n">
+        <v>1337758.74</v>
+      </c>
+      <c r="F129" s="40" t="n">
+        <v>-243134.06</v>
+      </c>
+      <c r="G129" s="40" t="n">
+        <v>-167596.64</v>
+      </c>
+      <c r="H129" s="7" t="n">
+        <v>0.051413</v>
+      </c>
+      <c r="I129" s="58" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="130"/>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>12. R7 DISTRESS PLAYBOOK (DOWNSIDE CASE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="59" t="inlineStr">
+        <is>
+          <t>THE LENDER IS REPAID ON SALE, BUT THE EQUITY IS WIPED OUT - DO NOT THROW A CURE AT A DEMAND FAILURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="133"/>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
+          <t>Minimum DSCR / year</t>
+        </is>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>0.79x in Year 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>Cumulative CFADS shortfall (EUR)</t>
+        </is>
+      </c>
+      <c r="B135" s="40" t="n">
+        <v>4577.04</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>Equity cure to 1.25x DSCR (EUR)</t>
+        </is>
+      </c>
+      <c r="B136" s="40" t="n">
+        <v>17455.75</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>Six-month DSRA (EUR)</t>
+        </is>
+      </c>
+      <c r="B137" s="40" t="n">
+        <v>20292.72</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="6" t="inlineStr">
+        <is>
+          <t>Net exit value (EUR)</t>
+        </is>
+      </c>
+      <c r="B138" s="40" t="n">
+        <v>654606.8199999999</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>Debt outstanding at exit (EUR)</t>
+        </is>
+      </c>
+      <c r="B139" s="40" t="n">
+        <v>457236.43</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>Lender recovery</t>
+        </is>
+      </c>
+      <c r="B140" s="56" t="n">
+        <v>1.4317</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>Equity at exit (EUR)</t>
+        </is>
+      </c>
+      <c r="B141" s="40" t="n">
+        <v>197370.39</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>Equity invested (EUR)</t>
+        </is>
+      </c>
+      <c r="B142" s="40" t="n">
+        <v>1113342.89</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>Equity recovery</t>
+        </is>
+      </c>
+      <c r="B143" s="56" t="n">
+        <v>0.1773</v>
+      </c>
+    </row>
+    <row r="144"/>
+    <row r="145">
+      <c r="A145" s="42" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B145" s="42" t="inlineStr">
+        <is>
+          <t>CFADS (EUR)</t>
+        </is>
+      </c>
+      <c r="C145" s="42" t="inlineStr">
+        <is>
+          <t>Debt service (EUR)</t>
+        </is>
+      </c>
+      <c r="D145" s="42" t="inlineStr">
+        <is>
+          <t>Shortfall (EUR)</t>
+        </is>
+      </c>
+      <c r="E145" s="42" t="inlineStr">
+        <is>
+          <t>DSCR</t>
+        </is>
+      </c>
+      <c r="F145" s="42" t="inlineStr">
+        <is>
+          <t>Ending cash (EUR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="B146" s="40" t="n">
+        <v>17004</v>
+      </c>
+      <c r="C146" s="40" t="n">
+        <v>21581.04</v>
+      </c>
+      <c r="D146" s="40" t="n">
+        <v>4577.04</v>
+      </c>
+      <c r="E146" s="43" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F146" s="40" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="B147" s="40" t="n">
+        <v>43248.35</v>
+      </c>
+      <c r="C147" s="40" t="n">
+        <v>40585.44</v>
+      </c>
+      <c r="D147" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" s="43" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F147" s="40" t="n">
+        <v>173204.5</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="B148" s="40" t="n">
+        <v>58730.24</v>
+      </c>
+      <c r="C148" s="40" t="n">
+        <v>40585.44</v>
+      </c>
+      <c r="D148" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" s="43" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F148" s="40" t="n">
+        <v>191349.3</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="B149" s="40" t="n">
+        <v>58730.24</v>
+      </c>
+      <c r="C149" s="40" t="n">
+        <v>40585.44</v>
+      </c>
+      <c r="D149" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" s="43" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F149" s="40" t="n">
+        <v>209494.1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="B150" s="40" t="n">
+        <v>58730.24</v>
+      </c>
+      <c r="C150" s="40" t="n">
+        <v>40585.44</v>
+      </c>
+      <c r="D150" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" s="43" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F150" s="40" t="n">
+        <v>227638.9</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="A77:N77"/>
     <mergeCell ref="A64:N64"/>
     <mergeCell ref="A73:N73"/>
     <mergeCell ref="A103:N103"/>
+    <mergeCell ref="A132:N132"/>
     <mergeCell ref="A70:N70"/>
     <mergeCell ref="A69:N69"/>
     <mergeCell ref="A65:N65"/>
+    <mergeCell ref="A108:N108"/>
     <mergeCell ref="A75:N75"/>
     <mergeCell ref="A66:N66"/>
     <mergeCell ref="A74:N74"/>

</xml_diff>